<commit_message>
Comparing smart chamber & SoilFluxPro
I exported a file containing both flux values from SoilFluxPro and the smart chamber to compare between them, and I exported a figure comparing them
</commit_message>
<xml_diff>
--- a/Data/Input/Soil gas efflux/2026/October/Clean/October 5, 2026 fluxes.xlsx
+++ b/Data/Input/Soil gas efflux/2026/October/Clean/October 5, 2026 fluxes.xlsx
@@ -604,14 +604,14 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Fluxes for both CO2 and methane have units of micromole per square</t>
+          <t>Fluxes for both CO2 are in either micromole (for CO2) or nanomole (for methane)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>meter per second. Soil area is in centimeter square while offset</t>
+          <t>per square meter per second. Soil area is in centimeter square while offset</t>
         </is>
       </c>
     </row>

</xml_diff>